<commit_message>
Update files for version 2.2
</commit_message>
<xml_diff>
--- a/product-definitions/spreadsheet/_vocabularies.xlsx
+++ b/product-definitions/spreadsheet/_vocabularies.xlsx
@@ -18,7 +18,7 @@
     <author/>
   </authors>
   <commentList>
-    <comment authorId="0" ref="A50">
+    <comment authorId="0" ref="A51">
       <text>
         <t xml:space="preserve">Need to add plot and photo which will be used in the NCAS Image standard v1.1
 	-sarah.hanrahan@stfc.ac.uk</t>
@@ -29,12 +29,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="160">
   <si>
     <t>Data Product</t>
   </si>
   <si>
     <t>acoustic-backscatter-winds</t>
+  </si>
+  <si>
+    <t>aerosol-backscatter-multi-wavelength</t>
   </si>
   <si>
     <t>aerosol-backscatter-radial-winds</t>
@@ -79,7 +82,7 @@
     <t>ch4-concentration</t>
   </si>
   <si>
-    <t>ch4-n2o-co-concentration</t>
+    <t>ch4-n2o-co2-co-concentration</t>
   </si>
   <si>
     <t>cloud-base</t>
@@ -197,6 +200,9 @@
   </si>
   <si>
     <t>radon-concentration</t>
+  </si>
+  <si>
+    <t>radon-radioactivity</t>
   </si>
   <si>
     <t>rain-lwc-velocity-reflectivity</t>
@@ -536,12 +542,10 @@
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -590,7 +594,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="18">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -601,19 +605,13 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
@@ -633,9 +631,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="top"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
@@ -920,7 +915,7 @@
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" s="4"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -942,10 +937,9 @@
       <c r="U3" s="2"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -1117,7 +1111,7 @@
       <c r="U10" s="2"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="2"/>
@@ -1142,7 +1136,7 @@
       <c r="U11" s="2"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B12" s="2"/>
@@ -1167,7 +1161,7 @@
       <c r="U12" s="2"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B13" s="2"/>
@@ -1192,7 +1186,7 @@
       <c r="U13" s="2"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B14" s="2"/>
@@ -1217,7 +1211,7 @@
       <c r="U14" s="2"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B15" s="2"/>
@@ -1292,7 +1286,7 @@
       <c r="U17" s="2"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>17</v>
       </c>
       <c r="B18" s="2"/>
@@ -1817,7 +1811,7 @@
       <c r="U38" s="2"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="6" t="s">
+      <c r="A39" s="3" t="s">
         <v>38</v>
       </c>
       <c r="B39" s="2"/>
@@ -1892,7 +1886,7 @@
       <c r="U41" s="2"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="6" t="s">
+      <c r="A42" s="3" t="s">
         <v>41</v>
       </c>
       <c r="B42" s="2"/>
@@ -1991,7 +1985,7 @@
       <c r="T45" s="2"/>
       <c r="U45" s="2"/>
     </row>
-    <row r="46" ht="15.0" customHeight="1">
+    <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="3" t="s">
         <v>45</v>
       </c>
@@ -2017,7 +2011,7 @@
       <c r="U46" s="2"/>
     </row>
     <row r="47" ht="15.0" customHeight="1">
-      <c r="A47" s="7" t="s">
+      <c r="A47" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B47" s="2"/>
@@ -2042,7 +2036,7 @@
       <c r="U47" s="2"/>
     </row>
     <row r="48" ht="15.0" customHeight="1">
-      <c r="A48" s="8" t="s">
+      <c r="A48" s="6" t="s">
         <v>47</v>
       </c>
       <c r="B48" s="2"/>
@@ -2066,8 +2060,8 @@
       <c r="T48" s="2"/>
       <c r="U48" s="2"/>
     </row>
-    <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="3" t="s">
+    <row r="49" ht="15.0" customHeight="1">
+      <c r="A49" s="6" t="s">
         <v>48</v>
       </c>
       <c r="B49" s="2"/>
@@ -2092,7 +2086,7 @@
       <c r="U49" s="2"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="3" t="s">
         <v>49</v>
       </c>
       <c r="B50" s="2"/>
@@ -2142,7 +2136,7 @@
       <c r="U51" s="2"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="6" t="s">
+      <c r="A52" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B52" s="2"/>
@@ -2167,7 +2161,7 @@
       <c r="U52" s="2"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="6" t="s">
+      <c r="A53" s="3" t="s">
         <v>52</v>
       </c>
       <c r="B53" s="2"/>
@@ -2242,7 +2236,7 @@
       <c r="U55" s="2"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="6" t="s">
+      <c r="A56" s="3" t="s">
         <v>55</v>
       </c>
       <c r="B56" s="2"/>
@@ -2292,7 +2286,7 @@
       <c r="U57" s="2"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="6" t="s">
+      <c r="A58" s="4" t="s">
         <v>57</v>
       </c>
       <c r="B58" s="2"/>
@@ -2467,7 +2461,7 @@
       <c r="U64" s="2"/>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="6" t="s">
+      <c r="A65" s="3" t="s">
         <v>64</v>
       </c>
       <c r="B65" s="2"/>
@@ -2567,7 +2561,9 @@
       <c r="U68" s="2"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="2"/>
+      <c r="A69" s="3" t="s">
+        <v>68</v>
+      </c>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
       <c r="D69" s="2"/>
@@ -2590,7 +2586,9 @@
       <c r="U69" s="2"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
-      <c r="A70" s="2"/>
+      <c r="A70" s="3" t="s">
+        <v>69</v>
+      </c>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
       <c r="D70" s="2"/>
@@ -7166,8 +7164,52 @@
       <c r="T268" s="2"/>
       <c r="U268" s="2"/>
     </row>
-    <row r="269" ht="15.75" customHeight="1"/>
-    <row r="270" ht="15.75" customHeight="1"/>
+    <row r="269" ht="15.75" customHeight="1">
+      <c r="A269" s="2"/>
+      <c r="B269" s="2"/>
+      <c r="C269" s="2"/>
+      <c r="D269" s="2"/>
+      <c r="E269" s="2"/>
+      <c r="F269" s="2"/>
+      <c r="G269" s="2"/>
+      <c r="H269" s="2"/>
+      <c r="I269" s="2"/>
+      <c r="J269" s="2"/>
+      <c r="K269" s="2"/>
+      <c r="L269" s="2"/>
+      <c r="M269" s="2"/>
+      <c r="N269" s="2"/>
+      <c r="O269" s="2"/>
+      <c r="P269" s="2"/>
+      <c r="Q269" s="2"/>
+      <c r="R269" s="2"/>
+      <c r="S269" s="2"/>
+      <c r="T269" s="2"/>
+      <c r="U269" s="2"/>
+    </row>
+    <row r="270" ht="15.75" customHeight="1">
+      <c r="A270" s="2"/>
+      <c r="B270" s="2"/>
+      <c r="C270" s="2"/>
+      <c r="D270" s="2"/>
+      <c r="E270" s="2"/>
+      <c r="F270" s="2"/>
+      <c r="G270" s="2"/>
+      <c r="H270" s="2"/>
+      <c r="I270" s="2"/>
+      <c r="J270" s="2"/>
+      <c r="K270" s="2"/>
+      <c r="L270" s="2"/>
+      <c r="M270" s="2"/>
+      <c r="N270" s="2"/>
+      <c r="O270" s="2"/>
+      <c r="P270" s="2"/>
+      <c r="Q270" s="2"/>
+      <c r="R270" s="2"/>
+      <c r="S270" s="2"/>
+      <c r="T270" s="2"/>
+      <c r="U270" s="2"/>
+    </row>
     <row r="271" ht="15.75" customHeight="1"/>
     <row r="272" ht="15.75" customHeight="1"/>
     <row r="273" ht="15.75" customHeight="1"/>
@@ -7900,14 +7942,6 @@
     <row r="1000" ht="15.75" customHeight="1"/>
     <row r="1001" ht="15.75" customHeight="1"/>
     <row r="1002" ht="15.75" customHeight="1"/>
-    <row r="1003" ht="15.75" customHeight="1"/>
-    <row r="1004" ht="15.75" customHeight="1"/>
-    <row r="1005" ht="15.75" customHeight="1"/>
-    <row r="1006" ht="15.75" customHeight="1"/>
-    <row r="1007" ht="15.75" customHeight="1"/>
-    <row r="1008" ht="15.75" customHeight="1"/>
-    <row r="1009" ht="15.75" customHeight="1"/>
-    <row r="1010" ht="15.75" customHeight="1"/>
   </sheetData>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
@@ -7928,233 +7962,233 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="C1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="B1" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="10"/>
-      <c r="Q1" s="10"/>
-      <c r="R1" s="10"/>
-      <c r="S1" s="10"/>
-      <c r="T1" s="10"/>
-      <c r="U1" s="10"/>
-      <c r="V1" s="10"/>
-      <c r="W1" s="10"/>
-      <c r="X1" s="10"/>
+      <c r="C1" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
+      <c r="R1" s="8"/>
+      <c r="S1" s="8"/>
+      <c r="T1" s="8"/>
+      <c r="U1" s="8"/>
+      <c r="V1" s="8"/>
+      <c r="W1" s="8"/>
+      <c r="X1" s="8"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="C2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="B2" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="E2" s="11"/>
+      <c r="C2" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="E2" s="9"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="B3" s="11" t="s">
+      <c r="A3" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" ht="15.75" customHeight="1">
+      <c r="A8" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="D15" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="13" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="C15" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>75</v>
-      </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="C16" s="15" t="s">
+      <c r="A16" s="9" t="s">
         <v>114</v>
       </c>
+      <c r="B16" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="C17" s="15" t="s">
+      <c r="A17" s="9" t="s">
         <v>117</v>
       </c>
+      <c r="B17" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="C18" s="15" t="s">
+      <c r="A18" s="9" t="s">
         <v>120</v>
       </c>
+      <c r="B18" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="C19" s="15" t="s">
+      <c r="A19" s="9" t="s">
         <v>123</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1"/>
@@ -9175,8 +9209,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="16" t="s">
-        <v>124</v>
+      <c r="A1" s="14" t="s">
+        <v>126</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -9231,20 +9265,20 @@
       <c r="Y2" s="2"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="C3" s="17" t="s">
+      <c r="A3" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="B3" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="C3" s="15" t="s">
         <v>129</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>131</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -9268,19 +9302,19 @@
       <c r="Y3" s="2"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="19" t="s">
-        <v>130</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
+      <c r="A4" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
@@ -9301,17 +9335,17 @@
       <c r="Y4" s="2"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="19"/>
-      <c r="B5" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
+      <c r="A5" s="5"/>
+      <c r="B5" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -9332,13 +9366,13 @@
       <c r="Y5" s="2"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="19"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
+      <c r="A6" s="5"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -9359,23 +9393,23 @@
       <c r="Y6" s="2"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="C7" s="19" t="s">
+      <c r="A7" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="B7" s="17" t="s">
         <v>136</v>
       </c>
+      <c r="C7" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>138</v>
+      </c>
       <c r="E7" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
+        <v>139</v>
+      </c>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -9396,19 +9430,19 @@
       <c r="Y7" s="2"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="19"/>
-      <c r="B8" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>138</v>
+      <c r="A8" s="5"/>
+      <c r="B8" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>140</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
+        <v>139</v>
+      </c>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -9429,19 +9463,19 @@
       <c r="Y8" s="2"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="19"/>
-      <c r="B9" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="C9" s="19" t="s">
+      <c r="A9" s="5"/>
+      <c r="B9" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -9462,19 +9496,19 @@
       <c r="Y9" s="2"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="19"/>
-      <c r="B10" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>140</v>
+      <c r="A10" s="5"/>
+      <c r="B10" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>142</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
+        <v>139</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -9495,19 +9529,19 @@
       <c r="Y10" s="2"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="19"/>
-      <c r="B11" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>141</v>
+      <c r="A11" s="5"/>
+      <c r="B11" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>143</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
+        <v>139</v>
+      </c>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -9528,19 +9562,19 @@
       <c r="Y11" s="2"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="19"/>
-      <c r="B12" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>142</v>
+      <c r="A12" s="5"/>
+      <c r="B12" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
+        <v>139</v>
+      </c>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -9561,19 +9595,19 @@
       <c r="Y12" s="2"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="19"/>
-      <c r="B13" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>143</v>
+      <c r="A13" s="5"/>
+      <c r="B13" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>145</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
+        <v>139</v>
+      </c>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
@@ -9594,19 +9628,19 @@
       <c r="Y13" s="2"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="19"/>
-      <c r="B14" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>144</v>
+      <c r="A14" s="5"/>
+      <c r="B14" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>146</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
+        <v>139</v>
+      </c>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -9628,14 +9662,14 @@
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="3"/>
-      <c r="B15" s="20" t="s">
-        <v>134</v>
+      <c r="B15" s="17" t="s">
+        <v>136</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -9687,14 +9721,14 @@
       <c r="Y16" s="2"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="19" t="s">
-        <v>133</v>
+      <c r="A17" s="5" t="s">
+        <v>135</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
@@ -9748,16 +9782,16 @@
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>150</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
@@ -9785,10 +9819,10 @@
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>148</v>
+        <v>151</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>150</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
@@ -9813,7 +9847,7 @@
       <c r="Y20" s="2"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="7"/>
+      <c r="A21" s="6"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -9840,14 +9874,14 @@
       <c r="Y21" s="2"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="7" t="s">
-        <v>150</v>
+      <c r="A22" s="6" t="s">
+        <v>152</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
@@ -9873,14 +9907,14 @@
       <c r="Y22" s="2"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="7" t="s">
-        <v>152</v>
+      <c r="A23" s="6" t="s">
+        <v>154</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
@@ -9906,14 +9940,14 @@
       <c r="Y23" s="2"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="7" t="s">
-        <v>154</v>
+      <c r="A24" s="6" t="s">
+        <v>156</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
@@ -9967,13 +10001,13 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>

</xml_diff>